<commit_message>
Actualización administrativa de inventario.xlsx (FerreteríaMS v0)
</commit_message>
<xml_diff>
--- a/03_Aplicacion/inventario.xlsx
+++ b/03_Aplicacion/inventario.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,6 +439,28 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Descripcion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>TEST001</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Martillo de prueba FerreteríaMS</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>CAT001</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Producto de evaluación del guardado GitHub API</t>
         </is>
       </c>
     </row>
@@ -637,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -657,6 +679,23 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>TEST001</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>U001</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>